<commit_message>
Removed block graph framework
</commit_message>
<xml_diff>
--- a/TrackModel/Green Line.xlsx
+++ b/TrackModel/Green Line.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pitt-my.sharepoint.com/personal/dgs44_pitt_edu/Documents/Trains/TrackModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="568" documentId="8_{D0660D75-C052-4898-8402-12AA78E71664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8C98194-8817-4F58-A7F3-D176B0B28C60}"/>
+  <xr:revisionPtr revIDLastSave="608" documentId="8_{D0660D75-C052-4898-8402-12AA78E71664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50BA1C67-8B17-4746-87A0-AC8F3AF98ADC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C71A2FFE-490E-4D57-BAA4-DE7AC575C897}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="73">
   <si>
     <t>A</t>
   </si>
@@ -218,10 +218,43 @@
     <t>Yard</t>
   </si>
   <si>
-    <t>adj1</t>
-  </si>
-  <si>
-    <t>adj2</t>
+    <t>Edgebrook,L</t>
+  </si>
+  <si>
+    <t>Whited,LR</t>
+  </si>
+  <si>
+    <t>Station,LR</t>
+  </si>
+  <si>
+    <t>South Bank,L</t>
+  </si>
+  <si>
+    <t>Central,R</t>
+  </si>
+  <si>
+    <t>Inglewood,R</t>
+  </si>
+  <si>
+    <t>Overbrook,R</t>
+  </si>
+  <si>
+    <t>Glenbury,R</t>
+  </si>
+  <si>
+    <t>Dormont,R</t>
+  </si>
+  <si>
+    <t>Mt Lebanon,LR</t>
+  </si>
+  <si>
+    <t>Poplar,L</t>
+  </si>
+  <si>
+    <t>Castle Shannon,L</t>
+  </si>
+  <si>
+    <t>Inglewood,L</t>
   </si>
 </sst>
 </file>
@@ -688,12 +721,6 @@
       <c r="S1" s="3">
         <v>18</v>
       </c>
-      <c r="T1" s="3">
-        <v>19</v>
-      </c>
-      <c r="U1" s="3">
-        <v>20</v>
-      </c>
     </row>
     <row r="2" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -752,12 +779,6 @@
       </c>
       <c r="S2" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:21" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -804,12 +825,8 @@
       <c r="S3" s="3">
         <v>11</v>
       </c>
-      <c r="T3" s="3">
-        <v>58</v>
-      </c>
-      <c r="U3" s="3">
-        <v>62</v>
-      </c>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
     </row>
     <row r="4" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -845,12 +862,6 @@
       </c>
       <c r="S4" s="3">
         <v>1</v>
-      </c>
-      <c r="T4" s="3">
-        <v>13</v>
-      </c>
-      <c r="U4" s="3">
-        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
@@ -890,12 +901,6 @@
         <f t="shared" si="0"/>
         <v>1.6</v>
       </c>
-      <c r="T5" s="3">
-        <v>1</v>
-      </c>
-      <c r="U5" s="3">
-        <v>3</v>
-      </c>
     </row>
     <row r="6" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -940,12 +945,6 @@
         <f t="shared" si="0"/>
         <v>2.2999999999999998</v>
       </c>
-      <c r="T6" s="3">
-        <v>2</v>
-      </c>
-      <c r="U6" s="3">
-        <v>4</v>
-      </c>
     </row>
     <row r="7" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -983,12 +982,6 @@
       <c r="S7" s="3">
         <f t="shared" si="0"/>
         <v>3</v>
-      </c>
-      <c r="T7" s="3">
-        <v>3</v>
-      </c>
-      <c r="U7" s="3">
-        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
@@ -1030,12 +1023,6 @@
         <f t="shared" si="0"/>
         <v>3.5</v>
       </c>
-      <c r="T8" s="3">
-        <v>4</v>
-      </c>
-      <c r="U8" s="3">
-        <v>6</v>
-      </c>
     </row>
     <row r="9" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -1076,12 +1063,6 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="T9" s="3">
-        <v>5</v>
-      </c>
-      <c r="U9" s="3">
-        <v>7</v>
-      </c>
     </row>
     <row r="10" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -1120,12 +1101,6 @@
         <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
-      <c r="T10" s="3">
-        <v>6</v>
-      </c>
-      <c r="U10" s="3">
-        <v>8</v>
-      </c>
     </row>
     <row r="11" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -1150,6 +1125,9 @@
       <c r="H11" s="2">
         <v>17</v>
       </c>
+      <c r="L11" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="P11" s="3">
         <v>18</v>
       </c>
@@ -1164,12 +1142,6 @@
         <f t="shared" ref="S11:S31" si="2">Q10</f>
         <v>4</v>
       </c>
-      <c r="T11" s="3">
-        <v>7</v>
-      </c>
-      <c r="U11" s="3">
-        <v>9</v>
-      </c>
     </row>
     <row r="12" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -1214,12 +1186,6 @@
         <f t="shared" ref="S12:S16" si="4">Q11</f>
         <v>2.5</v>
       </c>
-      <c r="T12" s="3">
-        <v>8</v>
-      </c>
-      <c r="U12" s="3">
-        <v>10</v>
-      </c>
     </row>
     <row r="13" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -1244,6 +1210,9 @@
       <c r="H13" s="2">
         <v>7.5</v>
       </c>
+      <c r="L13" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="P13" s="3">
         <v>14.5</v>
       </c>
@@ -1258,12 +1227,6 @@
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
-      <c r="T13" s="3">
-        <v>9</v>
-      </c>
-      <c r="U13" s="3">
-        <v>11</v>
-      </c>
     </row>
     <row r="14" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
@@ -1302,12 +1265,6 @@
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="T14" s="3">
-        <v>10</v>
-      </c>
-      <c r="U14" s="3">
-        <v>12</v>
-      </c>
     </row>
     <row r="15" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
@@ -1345,12 +1302,6 @@
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="T15" s="3">
-        <v>11</v>
-      </c>
-      <c r="U15" s="3">
-        <v>13</v>
-      </c>
     </row>
     <row r="16" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
@@ -1397,14 +1348,8 @@
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="T16" s="3">
-        <v>12</v>
-      </c>
-      <c r="U16" s="3">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -1443,14 +1388,8 @@
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="T17" s="3">
-        <v>13</v>
-      </c>
-      <c r="U17" s="3">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -1474,6 +1413,9 @@
       </c>
       <c r="H18" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="P18" s="3">
         <v>8</v>
@@ -1489,14 +1431,8 @@
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="T18" s="3">
-        <v>14</v>
-      </c>
-      <c r="U18" s="3">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -1541,14 +1477,8 @@
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="T19" s="3">
-        <v>15</v>
-      </c>
-      <c r="U19" s="3">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -1572,6 +1502,9 @@
       </c>
       <c r="H20" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="P20" s="3">
         <v>6</v>
@@ -1587,14 +1520,8 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="T20" s="3">
-        <v>16</v>
-      </c>
-      <c r="U20" s="3">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -1633,14 +1560,8 @@
         <f t="shared" si="2"/>
         <v>1.5</v>
       </c>
-      <c r="T21" s="3">
-        <v>17</v>
-      </c>
-      <c r="U21" s="3">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -1682,14 +1603,8 @@
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="T22" s="3">
-        <v>18</v>
-      </c>
-      <c r="U22" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -1728,14 +1643,8 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="T23" s="3">
-        <v>19</v>
-      </c>
-      <c r="U23" s="3">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -1759,6 +1668,9 @@
       </c>
       <c r="H24" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="P24" s="3">
         <f>P23</f>
@@ -1776,14 +1688,8 @@
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="T24" s="3">
-        <v>20</v>
-      </c>
-      <c r="U24" s="3">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -1830,14 +1736,8 @@
         <f t="shared" si="2"/>
         <v>4.5999999999999996</v>
       </c>
-      <c r="T25" s="3">
-        <v>21</v>
-      </c>
-      <c r="U25" s="3">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
@@ -1861,6 +1761,9 @@
       </c>
       <c r="H26" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="P26" s="3">
         <f t="shared" si="6"/>
@@ -1878,14 +1781,8 @@
         <f t="shared" si="2"/>
         <v>5.1999999999999993</v>
       </c>
-      <c r="T26" s="3">
-        <v>22</v>
-      </c>
-      <c r="U26" s="3">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
@@ -1926,14 +1823,8 @@
         <f t="shared" si="2"/>
         <v>5.7999999999999989</v>
       </c>
-      <c r="T27" s="3">
-        <v>23</v>
-      </c>
-      <c r="U27" s="3">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>20</v>
       </c>
@@ -1974,14 +1865,8 @@
         <f t="shared" si="2"/>
         <v>6.3999999999999986</v>
       </c>
-      <c r="T28" s="3">
-        <v>24</v>
-      </c>
-      <c r="U28" s="3">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
@@ -2022,14 +1907,8 @@
         <f t="shared" si="2"/>
         <v>6.9999999999999982</v>
       </c>
-      <c r="T29" s="3">
-        <v>25</v>
-      </c>
-      <c r="U29" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2070,14 +1949,8 @@
         <f t="shared" si="2"/>
         <v>7.5999999999999979</v>
       </c>
-      <c r="T30" s="3">
-        <v>26</v>
-      </c>
-      <c r="U30" s="3">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="31" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
@@ -2124,14 +1997,8 @@
         <f t="shared" si="2"/>
         <v>8.1999999999999975</v>
       </c>
-      <c r="T31" s="3">
-        <v>27</v>
-      </c>
-      <c r="U31" s="3">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>20</v>
       </c>
@@ -2169,14 +2036,8 @@
         <f>Q31+0.6</f>
         <v>9.3999999999999968</v>
       </c>
-      <c r="T32" s="3">
-        <v>28</v>
-      </c>
-      <c r="U32" s="3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
@@ -2197,6 +2058,9 @@
       </c>
       <c r="H33" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="P33" s="3">
         <f t="shared" ref="P33:P61" si="8">R32</f>
@@ -2214,14 +2078,8 @@
         <f t="shared" ref="S33:S35" si="10">S32+0.6</f>
         <v>9.9999999999999964</v>
       </c>
-      <c r="T33" s="3">
-        <v>29</v>
-      </c>
-      <c r="U33" s="3">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
@@ -2265,14 +2123,8 @@
         <f t="shared" si="10"/>
         <v>10.599999999999996</v>
       </c>
-      <c r="T34" s="3">
-        <v>30</v>
-      </c>
-      <c r="U34" s="3">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>20</v>
       </c>
@@ -2293,6 +2145,9 @@
       </c>
       <c r="H35" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="P35" s="3">
         <f t="shared" si="8"/>
@@ -2310,14 +2165,8 @@
         <f t="shared" si="10"/>
         <v>11.199999999999996</v>
       </c>
-      <c r="T35" s="3">
-        <v>31</v>
-      </c>
-      <c r="U35" s="3">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>20</v>
       </c>
@@ -2355,14 +2204,8 @@
         <f>S35+0.8</f>
         <v>11.999999999999996</v>
       </c>
-      <c r="T36" s="3">
-        <v>32</v>
-      </c>
-      <c r="U36" s="3">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>20</v>
       </c>
@@ -2400,14 +2243,8 @@
         <f t="shared" ref="S37:S38" si="12">S36+0.8</f>
         <v>12.799999999999997</v>
       </c>
-      <c r="T37" s="3">
-        <v>33</v>
-      </c>
-      <c r="U37" s="3">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="38" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
@@ -2445,14 +2282,8 @@
         <f t="shared" si="12"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T38" s="3">
-        <v>34</v>
-      </c>
-      <c r="U38" s="3">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>20</v>
       </c>
@@ -2493,14 +2324,8 @@
         <f>S38</f>
         <v>13.599999999999998</v>
       </c>
-      <c r="T39" s="3">
-        <v>35</v>
-      </c>
-      <c r="U39" s="3">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="40" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>20</v>
       </c>
@@ -2541,14 +2366,8 @@
         <f t="shared" ref="S40:S60" si="14">S39</f>
         <v>13.599999999999998</v>
       </c>
-      <c r="T40" s="3">
-        <v>36</v>
-      </c>
-      <c r="U40" s="3">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="41" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>20</v>
       </c>
@@ -2572,6 +2391,9 @@
       </c>
       <c r="I41" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L41" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="P41" s="3">
         <f t="shared" si="8"/>
@@ -2589,14 +2411,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T41" s="3">
-        <v>37</v>
-      </c>
-      <c r="U41" s="3">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="42" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>20</v>
       </c>
@@ -2643,14 +2459,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T42" s="3">
-        <v>38</v>
-      </c>
-      <c r="U42" s="3">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="43" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>20</v>
       </c>
@@ -2674,6 +2484,9 @@
       </c>
       <c r="I43" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L43" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="P43" s="3">
         <f t="shared" si="8"/>
@@ -2691,14 +2504,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T43" s="3">
-        <v>39</v>
-      </c>
-      <c r="U43" s="3">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="44" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>20</v>
       </c>
@@ -2739,14 +2546,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T44" s="3">
-        <v>40</v>
-      </c>
-      <c r="U44" s="3">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="45" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>20</v>
       </c>
@@ -2787,14 +2588,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T45" s="3">
-        <v>41</v>
-      </c>
-      <c r="U45" s="3">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="46" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>20</v>
       </c>
@@ -2835,14 +2630,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T46" s="3">
-        <v>42</v>
-      </c>
-      <c r="U46" s="3">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="47" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
@@ -2883,14 +2672,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T47" s="3">
-        <v>43</v>
-      </c>
-      <c r="U47" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="48" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>20</v>
       </c>
@@ -2931,14 +2714,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T48" s="3">
-        <v>44</v>
-      </c>
-      <c r="U48" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="49" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
@@ -2979,14 +2756,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T49" s="3">
-        <v>45</v>
-      </c>
-      <c r="U49" s="3">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="50" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
@@ -3010,6 +2781,9 @@
       </c>
       <c r="I50" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L50" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="P50" s="3">
         <f t="shared" si="8"/>
@@ -3027,14 +2801,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T50" s="3">
-        <v>46</v>
-      </c>
-      <c r="U50" s="3">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="51" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>20</v>
       </c>
@@ -3081,14 +2849,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T51" s="3">
-        <v>47</v>
-      </c>
-      <c r="U51" s="3">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="52" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>20</v>
       </c>
@@ -3112,6 +2874,9 @@
       </c>
       <c r="I52" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L52" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="P52" s="3">
         <f t="shared" si="8"/>
@@ -3129,14 +2894,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T52" s="3">
-        <v>48</v>
-      </c>
-      <c r="U52" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="53" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>20</v>
       </c>
@@ -3177,14 +2936,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T53" s="3">
-        <v>49</v>
-      </c>
-      <c r="U53" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="54" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>20</v>
       </c>
@@ -3225,14 +2978,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T54" s="3">
-        <v>50</v>
-      </c>
-      <c r="U54" s="3">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="55" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>20</v>
       </c>
@@ -3273,14 +3020,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T55" s="3">
-        <v>51</v>
-      </c>
-      <c r="U55" s="3">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="56" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>20</v>
       </c>
@@ -3321,14 +3062,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T56" s="3">
-        <v>52</v>
-      </c>
-      <c r="U56" s="3">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="57" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>20</v>
       </c>
@@ -3369,14 +3104,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T57" s="3">
-        <v>53</v>
-      </c>
-      <c r="U57" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="58" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>20</v>
       </c>
@@ -3417,14 +3146,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T58" s="3">
-        <v>54</v>
-      </c>
-      <c r="U58" s="3">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="59" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>20</v>
       </c>
@@ -3448,6 +3171,9 @@
       </c>
       <c r="I59" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L59" s="3" t="s">
+        <v>66</v>
       </c>
       <c r="P59" s="3">
         <f t="shared" si="8"/>
@@ -3465,14 +3191,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T59" s="3">
-        <v>55</v>
-      </c>
-      <c r="U59" s="3">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="60" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>20</v>
       </c>
@@ -3519,14 +3239,8 @@
         <f t="shared" si="14"/>
         <v>13.599999999999998</v>
       </c>
-      <c r="T60" s="3">
-        <v>56</v>
-      </c>
-      <c r="U60" s="3">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="61" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>20</v>
       </c>
@@ -3553,6 +3267,9 @@
       </c>
       <c r="K61" s="3">
         <v>57</v>
+      </c>
+      <c r="L61" s="3" t="s">
+        <v>66</v>
       </c>
       <c r="P61" s="3">
         <f t="shared" si="8"/>
@@ -3570,14 +3287,8 @@
         <f>S60+0.8</f>
         <v>14.399999999999999</v>
       </c>
-      <c r="T61" s="3">
-        <v>57</v>
-      </c>
-      <c r="U61" s="3">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="62" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>20</v>
       </c>
@@ -3615,14 +3326,8 @@
         <f t="shared" ref="S62:S65" si="18">S61+0.8</f>
         <v>15.2</v>
       </c>
-      <c r="T62" s="3">
-        <v>58</v>
-      </c>
-      <c r="U62" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="63" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>20</v>
       </c>
@@ -3660,14 +3365,8 @@
         <f t="shared" si="18"/>
         <v>16</v>
       </c>
-      <c r="T63" s="3">
-        <v>59</v>
-      </c>
-      <c r="U63" s="3">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="64" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>20</v>
       </c>
@@ -3705,14 +3404,8 @@
         <f t="shared" si="18"/>
         <v>16.8</v>
       </c>
-      <c r="T64" s="3">
-        <v>60</v>
-      </c>
-      <c r="U64" s="3">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="65" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>20</v>
       </c>
@@ -3756,14 +3449,8 @@
         <f t="shared" si="18"/>
         <v>17.600000000000001</v>
       </c>
-      <c r="T65" s="3">
-        <v>61</v>
-      </c>
-      <c r="U65" s="3">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="66" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>20</v>
       </c>
@@ -3801,14 +3488,8 @@
         <f>S65+1</f>
         <v>18.600000000000001</v>
       </c>
-      <c r="T66" s="3">
-        <v>62</v>
-      </c>
-      <c r="U66" s="3">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="67" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>20</v>
       </c>
@@ -3829,6 +3510,9 @@
       </c>
       <c r="H67" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L67" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="P67" s="3">
         <f t="shared" ref="P67:P130" si="19">R66</f>
@@ -3846,14 +3530,8 @@
         <f>S66+1</f>
         <v>19.600000000000001</v>
       </c>
-      <c r="T67" s="3">
-        <v>63</v>
-      </c>
-      <c r="U67" s="3">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="68" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>20</v>
       </c>
@@ -3897,14 +3575,8 @@
         <f>S65+4.2</f>
         <v>21.8</v>
       </c>
-      <c r="T68" s="3">
-        <v>64</v>
-      </c>
-      <c r="U68" s="3">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="69" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>20</v>
       </c>
@@ -3925,6 +3597,9 @@
       </c>
       <c r="H69" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L69" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="P69" s="3">
         <f t="shared" si="19"/>
@@ -3942,14 +3617,8 @@
         <f>S68+2.2</f>
         <v>24</v>
       </c>
-      <c r="T69" s="3">
-        <v>65</v>
-      </c>
-      <c r="U69" s="3">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="70" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>20</v>
       </c>
@@ -3987,14 +3656,8 @@
         <f>S69+1</f>
         <v>25</v>
       </c>
-      <c r="T70" s="3">
-        <v>66</v>
-      </c>
-      <c r="U70" s="3">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="71" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>20</v>
       </c>
@@ -4032,14 +3695,8 @@
         <f>S68+4.2</f>
         <v>26</v>
       </c>
-      <c r="T71" s="3">
-        <v>67</v>
-      </c>
-      <c r="U71" s="3">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="72" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>20</v>
       </c>
@@ -4077,14 +3734,8 @@
         <f>S71+1</f>
         <v>27</v>
       </c>
-      <c r="T72" s="3">
-        <v>68</v>
-      </c>
-      <c r="U72" s="3">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="73" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>20</v>
       </c>
@@ -4122,14 +3773,8 @@
         <f t="shared" ref="S73:S76" si="23">S72+1</f>
         <v>28</v>
       </c>
-      <c r="T73" s="3">
-        <v>69</v>
-      </c>
-      <c r="U73" s="3">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="74" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>20</v>
       </c>
@@ -4167,14 +3812,8 @@
         <f t="shared" si="23"/>
         <v>29</v>
       </c>
-      <c r="T74" s="3">
-        <v>70</v>
-      </c>
-      <c r="U74" s="3">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="75" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>20</v>
       </c>
@@ -4195,6 +3834,9 @@
       </c>
       <c r="H75" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L75" s="3" t="s">
+        <v>68</v>
       </c>
       <c r="P75" s="3">
         <f t="shared" si="19"/>
@@ -4212,14 +3854,8 @@
         <f t="shared" si="23"/>
         <v>30</v>
       </c>
-      <c r="T75" s="3">
-        <v>71</v>
-      </c>
-      <c r="U75" s="3">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="76" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>20</v>
       </c>
@@ -4263,14 +3899,8 @@
         <f t="shared" si="23"/>
         <v>31</v>
       </c>
-      <c r="T76" s="3">
-        <v>72</v>
-      </c>
-      <c r="U76" s="3">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="77" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>20</v>
       </c>
@@ -4294,6 +3924,9 @@
       </c>
       <c r="H77" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L77" s="3" t="s">
+        <v>68</v>
       </c>
       <c r="P77" s="3">
         <f t="shared" si="19"/>
@@ -4311,14 +3944,8 @@
         <f>S76</f>
         <v>31</v>
       </c>
-      <c r="T77" s="3">
-        <v>73</v>
-      </c>
-      <c r="U77" s="3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="78" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>20</v>
       </c>
@@ -4359,14 +3986,8 @@
         <f t="shared" ref="S78:S79" si="25">S77</f>
         <v>31</v>
       </c>
-      <c r="T78" s="3">
-        <v>74</v>
-      </c>
-      <c r="U78" s="3">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="79" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>20</v>
       </c>
@@ -4390,6 +4011,9 @@
       </c>
       <c r="H79" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L79" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="P79" s="3">
         <f t="shared" si="19"/>
@@ -4407,14 +4031,8 @@
         <f t="shared" si="25"/>
         <v>31</v>
       </c>
-      <c r="T79" s="3">
-        <v>75</v>
-      </c>
-      <c r="U79" s="3">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="80" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>20</v>
       </c>
@@ -4467,14 +4085,8 @@
         <f>S79</f>
         <v>31</v>
       </c>
-      <c r="T80" s="3">
-        <v>76</v>
-      </c>
-      <c r="U80" s="3">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="81" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>20</v>
       </c>
@@ -4498,6 +4110,9 @@
       </c>
       <c r="H81" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L81" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="P81" s="3">
         <f t="shared" si="19"/>
@@ -4515,14 +4130,8 @@
         <f t="shared" ref="S81:S88" si="27">S80</f>
         <v>31</v>
       </c>
-      <c r="T81" s="3">
-        <v>77</v>
-      </c>
-      <c r="U81" s="3">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="82" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>20</v>
       </c>
@@ -4563,14 +4172,8 @@
         <f t="shared" si="27"/>
         <v>31</v>
       </c>
-      <c r="T82" s="3">
-        <v>78</v>
-      </c>
-      <c r="U82" s="3">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="83" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>20</v>
       </c>
@@ -4611,14 +4214,8 @@
         <f t="shared" si="27"/>
         <v>31</v>
       </c>
-      <c r="T83" s="3">
-        <v>79</v>
-      </c>
-      <c r="U83" s="3">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="84" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>20</v>
       </c>
@@ -4659,14 +4256,8 @@
         <f t="shared" si="27"/>
         <v>31</v>
       </c>
-      <c r="T84" s="3">
-        <v>80</v>
-      </c>
-      <c r="U84" s="3">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="85" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>20</v>
       </c>
@@ -4707,14 +4298,8 @@
         <f t="shared" si="27"/>
         <v>31</v>
       </c>
-      <c r="T85" s="3">
-        <v>81</v>
-      </c>
-      <c r="U85" s="3">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="86" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>20</v>
       </c>
@@ -4755,14 +4340,8 @@
         <f t="shared" si="27"/>
         <v>31</v>
       </c>
-      <c r="T86" s="3">
-        <v>82</v>
-      </c>
-      <c r="U86" s="3">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="87" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>20</v>
       </c>
@@ -4803,14 +4382,8 @@
         <f t="shared" si="27"/>
         <v>31</v>
       </c>
-      <c r="T87" s="3">
-        <v>83</v>
-      </c>
-      <c r="U87" s="3">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="88" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>20</v>
       </c>
@@ -4857,14 +4430,8 @@
         <f t="shared" si="27"/>
         <v>31</v>
       </c>
-      <c r="T88" s="3">
-        <v>84</v>
-      </c>
-      <c r="U88" s="3">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="89" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>20</v>
       </c>
@@ -4905,14 +4472,8 @@
         <f>S88</f>
         <v>31</v>
       </c>
-      <c r="T89" s="3">
-        <v>85</v>
-      </c>
-      <c r="U89" s="3">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="90" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>20</v>
       </c>
@@ -4936,6 +4497,9 @@
       </c>
       <c r="H90" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L90" s="3" t="s">
+        <v>70</v>
       </c>
       <c r="P90" s="3">
         <f>R89</f>
@@ -4953,14 +4517,8 @@
         <f t="shared" ref="S90:S91" si="29">S89</f>
         <v>31</v>
       </c>
-      <c r="T90" s="3">
-        <v>86</v>
-      </c>
-      <c r="U90" s="3">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="91" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>20</v>
       </c>
@@ -5007,14 +4565,8 @@
         <f t="shared" si="29"/>
         <v>31</v>
       </c>
-      <c r="T91" s="3">
-        <v>87</v>
-      </c>
-      <c r="U91" s="3">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="92" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>20</v>
       </c>
@@ -5035,6 +4587,9 @@
       </c>
       <c r="H92" s="2">
         <v>0.125</v>
+      </c>
+      <c r="L92" s="3" t="s">
+        <v>70</v>
       </c>
       <c r="P92" s="3">
         <f t="shared" si="19"/>
@@ -5052,14 +4607,8 @@
         <f>S91-0.8</f>
         <v>30.2</v>
       </c>
-      <c r="T92" s="3">
-        <v>88</v>
-      </c>
-      <c r="U92" s="3">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="93" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="93" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>20</v>
       </c>
@@ -5097,14 +4646,8 @@
         <f t="shared" ref="S93:S97" si="31">S92-0.8</f>
         <v>29.4</v>
       </c>
-      <c r="T93" s="3">
-        <v>89</v>
-      </c>
-      <c r="U93" s="3">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="94" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>20</v>
       </c>
@@ -5142,14 +4685,8 @@
         <f t="shared" si="31"/>
         <v>28.599999999999998</v>
       </c>
-      <c r="T94" s="3">
-        <v>90</v>
-      </c>
-      <c r="U94" s="3">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="95" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>20</v>
       </c>
@@ -5187,14 +4724,8 @@
         <f t="shared" si="31"/>
         <v>27.799999999999997</v>
       </c>
-      <c r="T95" s="3">
-        <v>91</v>
-      </c>
-      <c r="U95" s="3">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="96" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>20</v>
       </c>
@@ -5232,14 +4763,8 @@
         <f t="shared" si="31"/>
         <v>26.999999999999996</v>
       </c>
-      <c r="T96" s="3">
-        <v>92</v>
-      </c>
-      <c r="U96" s="3">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="97" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>20</v>
       </c>
@@ -5277,14 +4802,8 @@
         <f t="shared" si="31"/>
         <v>26.199999999999996</v>
       </c>
-      <c r="T97" s="3">
-        <v>93</v>
-      </c>
-      <c r="U97" s="3">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="98" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>20</v>
       </c>
@@ -5305,6 +4824,9 @@
       </c>
       <c r="H98" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L98" s="3" t="s">
+        <v>71</v>
       </c>
       <c r="P98" s="3">
         <f t="shared" si="19"/>
@@ -5322,14 +4844,8 @@
         <f>S97+0.8</f>
         <v>26.999999999999996</v>
       </c>
-      <c r="T98" s="3">
-        <v>94</v>
-      </c>
-      <c r="U98" s="3">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="99" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>20</v>
       </c>
@@ -5373,14 +4889,8 @@
         <f t="shared" ref="S99:S100" si="33">S98+0.8</f>
         <v>27.799999999999997</v>
       </c>
-      <c r="T99" s="3">
-        <v>95</v>
-      </c>
-      <c r="U99" s="3">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="100" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="100" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>20</v>
       </c>
@@ -5401,6 +4911,9 @@
       </c>
       <c r="H100" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L100" s="3" t="s">
+        <v>71</v>
       </c>
       <c r="P100" s="3">
         <f t="shared" si="19"/>
@@ -5418,14 +4931,8 @@
         <f t="shared" si="33"/>
         <v>28.599999999999998</v>
       </c>
-      <c r="T100" s="3">
-        <v>96</v>
-      </c>
-      <c r="U100" s="3">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="101" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>20</v>
       </c>
@@ -5463,14 +4970,8 @@
         <f>S100+0.8</f>
         <v>29.4</v>
       </c>
-      <c r="T101" s="3">
-        <v>97</v>
-      </c>
-      <c r="U101" s="3">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="102" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="102" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>20</v>
       </c>
@@ -5508,14 +5009,8 @@
         <f t="shared" ref="S102:S103" si="35">S101+0.8</f>
         <v>30.2</v>
       </c>
-      <c r="T102" s="3">
-        <v>98</v>
-      </c>
-      <c r="U102" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="103" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="103" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>20</v>
       </c>
@@ -5553,14 +5048,8 @@
         <f t="shared" si="35"/>
         <v>31</v>
       </c>
-      <c r="T103" s="3">
-        <v>99</v>
-      </c>
-      <c r="U103" s="3">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="104" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="104" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>20</v>
       </c>
@@ -5594,14 +5083,8 @@
       <c r="S104" s="3">
         <v>29</v>
       </c>
-      <c r="T104" s="3">
-        <v>77</v>
-      </c>
-      <c r="U104" s="3">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="105" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="105" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>20</v>
       </c>
@@ -5637,14 +5120,8 @@
       <c r="S105" s="3">
         <v>29</v>
       </c>
-      <c r="T105" s="3">
-        <v>101</v>
-      </c>
-      <c r="U105" s="3">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="106" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="106" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>20</v>
       </c>
@@ -5680,14 +5157,8 @@
       <c r="S106" s="3">
         <v>29</v>
       </c>
-      <c r="T106" s="3">
-        <v>102</v>
-      </c>
-      <c r="U106" s="3">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="107" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="107" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>20</v>
       </c>
@@ -5708,6 +5179,9 @@
       </c>
       <c r="H107" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L107" s="3" t="s">
+        <v>68</v>
       </c>
       <c r="P107" s="3">
         <f t="shared" si="19"/>
@@ -5723,14 +5197,8 @@
       <c r="S107" s="3">
         <v>29</v>
       </c>
-      <c r="T107" s="3">
-        <v>103</v>
-      </c>
-      <c r="U107" s="3">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="108" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="108" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>20</v>
       </c>
@@ -5774,14 +5242,8 @@
         <f>S107-1</f>
         <v>28</v>
       </c>
-      <c r="T108" s="3">
-        <v>104</v>
-      </c>
-      <c r="U108" s="3">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="109" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="109" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>20</v>
       </c>
@@ -5802,6 +5264,9 @@
       </c>
       <c r="H109" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L109" s="3" t="s">
+        <v>68</v>
       </c>
       <c r="P109" s="3">
         <f t="shared" si="19"/>
@@ -5819,14 +5284,8 @@
         <f t="shared" ref="S109:S112" si="37">S108-1</f>
         <v>27</v>
       </c>
-      <c r="T109" s="3">
-        <v>105</v>
-      </c>
-      <c r="U109" s="3">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="110" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="110" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>20</v>
       </c>
@@ -5864,14 +5323,8 @@
         <f t="shared" si="37"/>
         <v>26</v>
       </c>
-      <c r="T110" s="3">
-        <v>106</v>
-      </c>
-      <c r="U110" s="3">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="111" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="111" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>20</v>
       </c>
@@ -5912,14 +5365,8 @@
         <f t="shared" si="37"/>
         <v>25</v>
       </c>
-      <c r="T111" s="3">
-        <v>107</v>
-      </c>
-      <c r="U111" s="3">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="112" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="112" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>20</v>
       </c>
@@ -5957,14 +5404,8 @@
         <f t="shared" si="37"/>
         <v>24</v>
       </c>
-      <c r="T112" s="3">
-        <v>108</v>
-      </c>
-      <c r="U112" s="3">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="113" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="113" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>20</v>
       </c>
@@ -6002,14 +5443,8 @@
         <f>S112-0.7</f>
         <v>23.3</v>
       </c>
-      <c r="T113" s="3">
-        <v>109</v>
-      </c>
-      <c r="U113" s="3">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="114" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="114" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>20</v>
       </c>
@@ -6047,14 +5482,8 @@
         <f t="shared" ref="S114:S119" si="39">S113-0.7</f>
         <v>22.6</v>
       </c>
-      <c r="T114" s="3">
-        <v>110</v>
-      </c>
-      <c r="U114" s="3">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="115" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="115" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>20</v>
       </c>
@@ -6092,14 +5521,8 @@
         <f t="shared" si="39"/>
         <v>21.900000000000002</v>
       </c>
-      <c r="T115" s="3">
-        <v>111</v>
-      </c>
-      <c r="U115" s="3">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="116" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="116" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>20</v>
       </c>
@@ -6120,6 +5543,9 @@
       </c>
       <c r="H116" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L116" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="P116" s="3">
         <f t="shared" si="19"/>
@@ -6137,14 +5563,8 @@
         <f t="shared" si="39"/>
         <v>21.200000000000003</v>
       </c>
-      <c r="T116" s="3">
-        <v>112</v>
-      </c>
-      <c r="U116" s="3">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="117" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="117" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>20</v>
       </c>
@@ -6188,14 +5608,8 @@
         <f t="shared" si="39"/>
         <v>20.500000000000004</v>
       </c>
-      <c r="T117" s="3">
-        <v>113</v>
-      </c>
-      <c r="U117" s="3">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="118" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="118" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>20</v>
       </c>
@@ -6216,6 +5630,9 @@
       </c>
       <c r="H118" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L118" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="P118" s="3">
         <f t="shared" si="19"/>
@@ -6233,14 +5650,8 @@
         <f t="shared" si="39"/>
         <v>19.800000000000004</v>
       </c>
-      <c r="T118" s="3">
-        <v>114</v>
-      </c>
-      <c r="U118" s="3">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="119" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="119" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>20</v>
       </c>
@@ -6278,14 +5689,8 @@
         <f t="shared" si="39"/>
         <v>19.100000000000005</v>
       </c>
-      <c r="T119" s="3">
-        <v>115</v>
-      </c>
-      <c r="U119" s="3">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="120" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="120" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>20</v>
       </c>
@@ -6323,14 +5728,8 @@
         <f>S119-0.8</f>
         <v>18.300000000000004</v>
       </c>
-      <c r="T120" s="3">
-        <v>116</v>
-      </c>
-      <c r="U120" s="3">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="121" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="121" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>20</v>
       </c>
@@ -6368,14 +5767,8 @@
         <f t="shared" ref="S121:S124" si="40">S120-0.8</f>
         <v>17.500000000000004</v>
       </c>
-      <c r="T121" s="3">
-        <v>117</v>
-      </c>
-      <c r="U121" s="3">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="122" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="122" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>20</v>
       </c>
@@ -6413,14 +5806,8 @@
         <f t="shared" si="40"/>
         <v>16.700000000000003</v>
       </c>
-      <c r="T122" s="3">
-        <v>118</v>
-      </c>
-      <c r="U122" s="3">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="123" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="123" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>20</v>
       </c>
@@ -6458,14 +5845,8 @@
         <f t="shared" si="40"/>
         <v>15.900000000000002</v>
       </c>
-      <c r="T123" s="3">
-        <v>119</v>
-      </c>
-      <c r="U123" s="3">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="124" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="124" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>20</v>
       </c>
@@ -6503,14 +5884,8 @@
         <f t="shared" si="40"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T124" s="3">
-        <v>120</v>
-      </c>
-      <c r="U124" s="3">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="125" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="125" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>20</v>
       </c>
@@ -6534,6 +5909,9 @@
       </c>
       <c r="I125" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L125" s="3" t="s">
+        <v>66</v>
       </c>
       <c r="P125" s="3">
         <f t="shared" si="19"/>
@@ -6551,14 +5929,8 @@
         <f>S124</f>
         <v>15.100000000000001</v>
       </c>
-      <c r="T125" s="3">
-        <v>121</v>
-      </c>
-      <c r="U125" s="3">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="126" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="126" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>20</v>
       </c>
@@ -6605,14 +5977,8 @@
         <f t="shared" ref="S126:S146" si="43">S125</f>
         <v>15.100000000000001</v>
       </c>
-      <c r="T126" s="3">
-        <v>122</v>
-      </c>
-      <c r="U126" s="3">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="127" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="127" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>20</v>
       </c>
@@ -6636,6 +6002,9 @@
       </c>
       <c r="I127" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L127" s="3" t="s">
+        <v>66</v>
       </c>
       <c r="P127" s="3">
         <f t="shared" si="19"/>
@@ -6653,14 +6022,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T127" s="3">
-        <v>123</v>
-      </c>
-      <c r="U127" s="3">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="128" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="128" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>20</v>
       </c>
@@ -6701,14 +6064,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T128" s="3">
-        <v>124</v>
-      </c>
-      <c r="U128" s="3">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="129" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="129" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>20</v>
       </c>
@@ -6749,14 +6106,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T129" s="3">
-        <v>125</v>
-      </c>
-      <c r="U129" s="3">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="130" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="130" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>20</v>
       </c>
@@ -6797,14 +6148,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T130" s="3">
-        <v>126</v>
-      </c>
-      <c r="U130" s="3">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="131" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="131" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>20</v>
       </c>
@@ -6845,14 +6190,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T131" s="3">
-        <v>127</v>
-      </c>
-      <c r="U131" s="3">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="132" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="132" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>20</v>
       </c>
@@ -6893,14 +6232,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T132" s="3">
-        <v>128</v>
-      </c>
-      <c r="U132" s="3">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="133" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="133" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>20</v>
       </c>
@@ -6941,14 +6274,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T133" s="3">
-        <v>129</v>
-      </c>
-      <c r="U133" s="3">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="134" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="134" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>20</v>
       </c>
@@ -6972,6 +6299,9 @@
       </c>
       <c r="I134" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L134" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="P134" s="3">
         <f t="shared" si="44"/>
@@ -6989,14 +6319,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T134" s="3">
-        <v>130</v>
-      </c>
-      <c r="U134" s="3">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="135" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="135" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>20</v>
       </c>
@@ -7043,14 +6367,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T135" s="3">
-        <v>131</v>
-      </c>
-      <c r="U135" s="3">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="136" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="136" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>20</v>
       </c>
@@ -7074,6 +6392,9 @@
       </c>
       <c r="I136" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L136" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="P136" s="3">
         <f t="shared" si="44"/>
@@ -7091,14 +6412,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T136" s="3">
-        <v>132</v>
-      </c>
-      <c r="U136" s="3">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="137" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="137" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>20</v>
       </c>
@@ -7139,14 +6454,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T137" s="3">
-        <v>133</v>
-      </c>
-      <c r="U137" s="3">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="138" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="138" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>20</v>
       </c>
@@ -7187,14 +6496,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T138" s="3">
-        <v>134</v>
-      </c>
-      <c r="U138" s="3">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="139" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="139" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>20</v>
       </c>
@@ -7235,14 +6538,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T139" s="3">
-        <v>135</v>
-      </c>
-      <c r="U139" s="3">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="140" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="140" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>20</v>
       </c>
@@ -7283,14 +6580,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T140" s="3">
-        <v>136</v>
-      </c>
-      <c r="U140" s="3">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="141" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="141" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>20</v>
       </c>
@@ -7331,14 +6622,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T141" s="3">
-        <v>137</v>
-      </c>
-      <c r="U141" s="3">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="142" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="142" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>20</v>
       </c>
@@ -7379,14 +6664,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T142" s="3">
-        <v>138</v>
-      </c>
-      <c r="U142" s="3">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="143" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="143" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>20</v>
       </c>
@@ -7410,6 +6689,9 @@
       </c>
       <c r="I143" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L143" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="P143" s="3">
         <f t="shared" si="44"/>
@@ -7427,14 +6709,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T143" s="3">
-        <v>139</v>
-      </c>
-      <c r="U143" s="3">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="144" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="144" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>20</v>
       </c>
@@ -7481,14 +6757,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T144" s="3">
-        <v>140</v>
-      </c>
-      <c r="U144" s="3">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="145" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="145" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>20</v>
       </c>
@@ -7512,6 +6782,9 @@
       </c>
       <c r="I145" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="L145" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="P145" s="3">
         <f t="shared" si="44"/>
@@ -7529,14 +6802,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T145" s="3">
-        <v>141</v>
-      </c>
-      <c r="U145" s="3">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="146" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="146" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>20</v>
       </c>
@@ -7577,14 +6844,8 @@
         <f t="shared" si="43"/>
         <v>15.100000000000001</v>
       </c>
-      <c r="T146" s="3">
-        <v>142</v>
-      </c>
-      <c r="U146" s="3">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="147" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="147" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>20</v>
       </c>
@@ -7622,14 +6883,8 @@
         <f>S146-0.7</f>
         <v>14.400000000000002</v>
       </c>
-      <c r="T147" s="3">
-        <v>143</v>
-      </c>
-      <c r="U147" s="3">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="148" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="148" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>20</v>
       </c>
@@ -7667,14 +6922,8 @@
         <f t="shared" ref="S148:S149" si="47">S147-0.7</f>
         <v>13.700000000000003</v>
       </c>
-      <c r="T148" s="3">
-        <v>144</v>
-      </c>
-      <c r="U148" s="3">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="149" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="149" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>20</v>
       </c>
@@ -7712,14 +6961,8 @@
         <f t="shared" si="47"/>
         <v>13.000000000000004</v>
       </c>
-      <c r="T149" s="3">
-        <v>145</v>
-      </c>
-      <c r="U149" s="3">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="150" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="150" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>20</v>
       </c>
@@ -7757,14 +7000,8 @@
         <f>S149-0.8</f>
         <v>12.200000000000003</v>
       </c>
-      <c r="T150" s="3">
-        <v>146</v>
-      </c>
-      <c r="U150" s="3">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="151" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="151" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>20</v>
       </c>
@@ -7802,14 +7039,8 @@
         <f t="shared" ref="S151:S152" si="49">S150-0.8</f>
         <v>11.400000000000002</v>
       </c>
-      <c r="T151" s="3">
-        <v>147</v>
-      </c>
-      <c r="U151" s="3">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="152" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="152" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>20</v>
       </c>
@@ -7847,14 +7078,8 @@
         <f t="shared" si="49"/>
         <v>10.600000000000001</v>
       </c>
-      <c r="T152" s="3">
-        <v>148</v>
-      </c>
-      <c r="U152" s="3">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="153" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="153" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>20</v>
       </c>
@@ -7890,17 +7115,11 @@
       <c r="S153" s="3">
         <v>8.8000000000000007</v>
       </c>
-      <c r="T153" s="3">
-        <v>149</v>
-      </c>
-      <c r="U153" s="3">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="155" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="155" spans="1:19" x14ac:dyDescent="0.25">
       <c r="H155"/>
     </row>
-    <row r="156" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:19" x14ac:dyDescent="0.25">
       <c r="H156"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
block occuipes one at a time, block 63 still fixed on instantiation, also the first station has beacons now
</commit_message>
<xml_diff>
--- a/TrackModel/Green Line.xlsx
+++ b/TrackModel/Green Line.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pitt-my.sharepoint.com/personal/dgs44_pitt_edu/Documents/Trains/TrackModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="680" documentId="8_{D0660D75-C052-4898-8402-12AA78E71664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6B8BD8C-0824-4FB3-96FB-EC0CF953EC59}"/>
+  <xr:revisionPtr revIDLastSave="682" documentId="8_{D0660D75-C052-4898-8402-12AA78E71664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE4F6CF7-A6F0-49F6-9AFB-C0390E7FA6A8}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{C71A2FFE-490E-4D57-BAA4-DE7AC575C897}"/>
+    <workbookView minimized="1" xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11295" xr2:uid="{C71A2FFE-490E-4D57-BAA4-DE7AC575C897}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="76">
   <si>
     <t>A</t>
   </si>
@@ -343,10 +343,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3532,6 +3528,9 @@
       <c r="H67" s="2">
         <v>0.5</v>
       </c>
+      <c r="L67" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P67" s="3">
         <f t="shared" ref="P67:P130" si="19">R66</f>
         <v>22.6</v>
@@ -3615,6 +3614,9 @@
       </c>
       <c r="H69" s="2">
         <v>0.5</v>
+      </c>
+      <c r="L69" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="P69" s="3">
         <f t="shared" si="19"/>

</xml_diff>